<commit_message>
[feat] 영웅 질환 UI List<string>으로 변경
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/HeroBasic.xlsx
+++ b/JsonConverter/ExcelFiles/HeroBasic.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="15765" windowHeight="4245"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="28545" windowHeight="11745"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="HeroBasic" sheetId="1" r:id="rId4"/>
@@ -19,15 +19,168 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="70">
+  <x:si>
+    <x:t>Frozen Widow</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CandidateWeight</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_01_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ProfileImage</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_04_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_07_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_03_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_06_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_02_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scarlet Twitch</x:t>
+  </x:si>
+  <x:si>
+    <x:t>heroSkill_05_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>질환</x:t>
+  </x:si>
+  <x:si>
+    <x:t>67세</x:t>
+  </x:si>
+  <x:si>
+    <x:t>50세</x:t>
+  </x:si>
+  <x:si>
+    <x:t>83세</x:t>
+  </x:si>
+  <x:si>
+    <x:t>88세</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나이</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Age</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>또르르</x:t>
+  </x:si>
+  <x:si>
+    <x:t>penalty_02,penalty_03,penalty_04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>냉기보다 오십견이 더 무서움. 팔을 높이 들면 표정이 급격히 차가워짐.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>방패를 베개처럼 끌어안고 잠. 회의가 길어지면 영웅담이 자동 재생됨.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>작은 글씨를 못 봄. 표적판보다 돋보기를 먼저 찾는 원거리 담당.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나이 미상</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Remarks</x:t>
+  </x:si>
+  <x:si>
+    <x:t>수령 732년</x:t>
+  </x:si>
+  <x:si>
+    <x:t>대표 스킬ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Groan</x:t>
+  </x:si>
+  <x:si>
+    <x:t>등장가중치</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스칼렛트위치</x:t>
+  </x:si>
+  <x:si>
+    <x:t>영웅 이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캡틴물렁카</x:t>
+  </x:si>
+  <x:si>
+    <x:t>약 1500세</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>호크아이고</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고목영감</x:t>
+  </x:si>
+  <x:si>
+    <x:t>할매프로스트</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_07</x:t>
+  </x:si>
+  <x:si>
+    <x:t>특이사항</x:t>
+  </x:si>
+  <x:si>
+    <x:t>영웅ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>프로필이미지</x:t>
+  </x:si>
+  <x:si>
+    <x:t>오십위도우</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hero_02</x:t>
+  </x:si>
   <x:si>
     <x:t>PenaltyID</x:t>
   </x:si>
   <x:si>
-    <x:t>penalty_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>penalty_02</x:t>
+    <x:t>penalty_06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>penalty_04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>penalty_05</x:t>
   </x:si>
   <x:si>
     <x:t>penalty_03</x:t>
@@ -36,196 +189,46 @@
     <x:t>penalty_07</x:t>
   </x:si>
   <x:si>
-    <x:t>penalty_04</x:t>
-  </x:si>
-  <x:si>
-    <x:t>penalty_05</x:t>
-  </x:si>
-  <x:si>
-    <x:t>penalty_06</x:t>
-  </x:si>
-  <x:si>
-    <x:t>67세</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나이</x:t>
-  </x:si>
-  <x:si>
-    <x:t>50세</x:t>
-  </x:si>
-  <x:si>
-    <x:t>또르르</x:t>
-  </x:si>
-  <x:si>
-    <x:t>88세</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>83세</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Age</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ID</x:t>
+    <x:t>MainSkillId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HeroNameEn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tinnitor</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HeroName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Squinteye</x:t>
+  </x:si>
+  <x:si>
+    <x:t>영웅 영문 이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Captain Mushmerica</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Granny Frostbite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>천둥 소리보다 관절 소리가 먼저 남. 망치를 자주 놓침.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>햇빛 좋은 곳을 선호함. 대화 중에도 가끔 잎이 떨어짐.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>감정 기복이 공간을 흔듦. 집중하면 주변 사물이 살짝 떨림.</x:t>
   </x:si>
   <x:si>
     <x:t>피부가 단단해지는 대신 간식 취향도 단단함. 아몬드를 늘 챙김.</x:t>
   </x:si>
   <x:si>
-    <x:t>감정 기복이 공간을 흔듦. 집중하면 주변 사물이 살짝 떨림.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>질환</x:t>
-  </x:si>
-  <x:si>
-    <x:t>냉기보다 오십견이 더 무서움. 팔을 높이 들면 표정이 급격히 차가워짐.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>작은 글씨를 못 봄. 표적판보다 돋보기를 먼저 찾는 원거리 담당.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>방패를 베개처럼 끌어안고 잠. 회의가 길어지면 영웅담이 자동 재생됨.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_05_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_07_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_04_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Frozen Widow</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_03_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ProfileImage</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_01_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_06_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>heroSkill_02_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CandidateWeight</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scarlet Twitch</x:t>
-  </x:si>
-  <x:si>
-    <x:t>천둥 소리보다 관절 소리가 먼저 남. 망치를 자주 놓침.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>햇빛 좋은 곳을 선호함. 대화 중에도 가끔 잎이 떨어짐.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>오십위도우</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>등장가중치</x:t>
-  </x:si>
-  <x:si>
-    <x:t>스칼렛트위치</x:t>
-  </x:si>
-  <x:si>
-    <x:t>영웅 이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>대표 스킬ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>특이사항</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Groan</x:t>
-  </x:si>
-  <x:si>
-    <x:t>할매프로스트</x:t>
-  </x:si>
-  <x:si>
-    <x:t>영웅ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>프로필이미지</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_07</x:t>
-  </x:si>
-  <x:si>
-    <x:t>약 1500세</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_06</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고목영감</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_04</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나이 미상</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Remarks</x:t>
-  </x:si>
-  <x:si>
-    <x:t>수령 732년</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캡틴물렁카</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hero_05</x:t>
-  </x:si>
-  <x:si>
-    <x:t>호크아이고</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HeroName</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MainSkillId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tinnitor</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Squinteye</x:t>
-  </x:si>
-  <x:si>
-    <x:t>영웅 영문 이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HeroNameEn</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Captain Mushmerica</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Granny Frostbite</x:t>
+    <x:t>penalty_01,penalty_02,penalty_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string[]</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1041,121 +1044,123 @@
     <x:col min="5" max="5" width="30.5703125" style="3" customWidth="1"/>
     <x:col min="6" max="6" width="26.5703125" style="3" customWidth="1"/>
     <x:col min="7" max="7" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <x:col min="8" max="16384" width="12.5703125" style="3"/>
+    <x:col min="8" max="8" width="12.5703125" style="3"/>
+    <x:col min="9" max="9" width="64.71484375" style="3" customWidth="1"/>
+    <x:col min="10" max="16384" width="12.5703125" style="3"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="C1" s="1" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="s">
-        <x:v>42</x:v>
-      </x:c>
       <x:c r="F1" s="3" t="s">
-        <x:v>41</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G1" s="3" t="s">
-        <x:v>38</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="H1" s="3" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="I1" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>55</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>55</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9" s="13" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="12" t="s">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B3" s="12" t="s">
-        <x:v>61</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C3" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E3" s="14" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F3" s="15" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="F3" s="15" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>32</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>28</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I3" s="13" t="s">
-        <x:v>0</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A4" s="4" t="s">
-        <x:v>49</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B4" s="4" t="s">
-        <x:v>58</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
-        <x:v>67</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D4" s="16" t="s">
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E4" s="16" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F4" s="17" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5" t="s">
-        <x:v>1</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J4" s="5"/>
       <x:c r="K4" s="5"/>
@@ -1166,29 +1171,29 @@
     </x:row>
     <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A5" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>36</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>26</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="16" t="s">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E5" s="16" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F5" s="16" t="s">
-        <x:v>31</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G5" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5" t="s">
-        <x:v>2</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="J5" s="5"/>
       <x:c r="K5" s="5"/>
@@ -1199,29 +1204,29 @@
     </x:row>
     <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A6" s="4" t="s">
-        <x:v>50</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C6" s="6" t="s">
-        <x:v>64</x:v>
-      </x:c>
       <x:c r="D6" s="16" t="s">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E6" s="16" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F6" s="16" t="s">
-        <x:v>27</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G6" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5" t="s">
-        <x:v>3</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="J6" s="5"/>
       <x:c r="K6" s="5"/>
@@ -1232,29 +1237,29 @@
     </x:row>
     <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A7" s="4" t="s">
-        <x:v>53</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B7" s="4" t="s">
-        <x:v>39</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C7" s="4" t="s">
-        <x:v>33</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D7" s="16" t="s">
-        <x:v>54</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E7" s="16" t="s">
-        <x:v>18</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F7" s="16" t="s">
-        <x:v>25</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G7" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5" t="s">
-        <x:v>5</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>
@@ -1265,29 +1270,29 @@
     </x:row>
     <x:row r="8" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A8" s="4" t="s">
-        <x:v>59</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>11</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
-        <x:v>63</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D8" s="16" t="s">
-        <x:v>48</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E8" s="16" t="s">
-        <x:v>34</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F8" s="16" t="s">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5" t="s">
-        <x:v>6</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="J8" s="5"/>
       <x:c r="K8" s="5"/>
@@ -1298,29 +1303,29 @@
     </x:row>
     <x:row r="9" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A9" s="4" t="s">
-        <x:v>51</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>52</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>43</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D9" s="16" t="s">
-        <x:v>57</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E9" s="16" t="s">
-        <x:v>35</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F9" s="16" t="s">
-        <x:v>30</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G9" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5" t="s">
-        <x:v>7</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="J9" s="5"/>
       <x:c r="K9" s="5"/>
@@ -1331,29 +1336,29 @@
     </x:row>
     <x:row r="10" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A10" s="4" t="s">
-        <x:v>47</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>68</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D10" s="16" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E10" s="16" t="s">
-        <x:v>17</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F10" s="16" t="s">
-        <x:v>24</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="5">
         <x:v>100</x:v>
       </x:c>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5" t="s">
-        <x:v>4</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="J10" s="5"/>
       <x:c r="K10" s="5"/>

</xml_diff>